<commit_message>
Modified topic wise Question Banks as standardized for adding in the app
</commit_message>
<xml_diff>
--- a/ASTquizApp/qBanks/DLI.xlsx
+++ b/ASTquizApp/qBanks/DLI.xlsx
@@ -1,15 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26626"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\programDo\vs\ASTquizApp\ASTquizApp\qBanks\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564DCA68-4590-4EE0-A711-F0B7F1BB5B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="0"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="12210" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$O$48</definedName>
@@ -19,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="152" count="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="152">
   <si>
     <t>Answer</t>
   </si>
@@ -513,40 +517,37 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6">
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b/>
       <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <name val="Arial"/>
       <sz val="12"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
     </font>
     <font>
+      <sz val="12"/>
       <name val="Arial"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="2">
@@ -590,55 +591,55 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C6500"/>
@@ -659,25 +660,23 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16" count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -715,7 +714,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -749,6 +748,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -783,9 +783,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -891,7 +892,7 @@
             <a:camera prst="orthographicFront">
               <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
+            <a:lightRig rig="threePt" dir="t">
               <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
@@ -958,28 +959,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P48"/>
-  <sheetFormatPr defaultRowHeight="15.0" defaultColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O48"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" hidden="1" customWidth="1" width="16.855469" style="0"/>
-    <col min="2" max="2" hidden="1" customWidth="1" bestFit="1" width="13.855469" style="0"/>
-    <col min="3" max="3" hidden="1" customWidth="1" bestFit="1" width="6.7109375" style="0"/>
-    <col min="4" max="4" hidden="1" customWidth="1" bestFit="1" width="7.2851562" style="0"/>
-    <col min="5" max="5" hidden="1" customWidth="1" bestFit="1" width="6.5703125" style="0"/>
-    <col min="6" max="6" hidden="1" customWidth="1" bestFit="1" width="10.0" style="0"/>
-    <col min="7" max="7" customWidth="1" bestFit="1" width="10.0" style="0"/>
-    <col min="8" max="8" customWidth="1" width="43.710938" style="0"/>
-    <col min="9" max="9" customWidth="1" bestFit="1" width="11.855469" style="0"/>
-    <col min="10" max="10" customWidth="1" width="13.855469" style="0"/>
-    <col min="11" max="11" customWidth="1" width="13.425781" style="0"/>
-    <col min="12" max="12" customWidth="1" width="12.285156" style="0"/>
-    <col min="13" max="13" customWidth="1" width="9.855469" style="0"/>
-    <col min="14" max="14" hidden="1" customWidth="1" bestFit="1" width="10.0" style="0"/>
-    <col min="15" max="15" hidden="1" customWidth="1" bestFit="1" width="18.710938" style="0"/>
+    <col min="1" max="1" width="67.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="65.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="8:8" s="1" ht="18.75" customFormat="1">
+    <row r="1" spans="1:15" s="1" customFormat="1" ht="18.75">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="2" spans="1:15" s="3" customFormat="1" ht="60">
       <c r="A2" s="4" t="s">
         <v>141</v>
       </c>
@@ -1034,7 +1034,7 @@
         <v>102</v>
       </c>
       <c r="C2" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>15</v>
@@ -1043,7 +1043,7 @@
         <v>21</v>
       </c>
       <c r="F2" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>140</v>
@@ -1067,13 +1067,13 @@
         <v>21</v>
       </c>
       <c r="N2" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O2" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="3" spans="1:15" s="3" customFormat="1" ht="45">
       <c r="A3" s="4" t="s">
         <v>141</v>
       </c>
@@ -1081,7 +1081,7 @@
         <v>102</v>
       </c>
       <c r="C3" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>15</v>
@@ -1090,7 +1090,7 @@
         <v>38</v>
       </c>
       <c r="F3" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>140</v>
@@ -1114,13 +1114,13 @@
         <v>28</v>
       </c>
       <c r="N3" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O3" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="4" spans="1:15" s="3" customFormat="1" ht="60">
       <c r="A4" s="4" t="s">
         <v>141</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>102</v>
       </c>
       <c r="C4" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>15</v>
@@ -1137,7 +1137,7 @@
         <v>36</v>
       </c>
       <c r="F4" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>139</v>
@@ -1157,13 +1157,13 @@
         <v>21</v>
       </c>
       <c r="N4" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O4" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="5" spans="1:15" s="3" customFormat="1" ht="60">
       <c r="A5" s="4" t="s">
         <v>141</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>102</v>
       </c>
       <c r="C5" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>15</v>
@@ -1180,7 +1180,7 @@
         <v>38</v>
       </c>
       <c r="F5" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>140</v>
@@ -1204,13 +1204,13 @@
         <v>21</v>
       </c>
       <c r="N5" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O5" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="6" spans="1:15" s="3" customFormat="1" ht="60">
       <c r="A6" s="4" t="s">
         <v>141</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>102</v>
       </c>
       <c r="C6" s="5">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>15</v>
@@ -1227,7 +1227,7 @@
         <v>38</v>
       </c>
       <c r="F6" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>140</v>
@@ -1251,13 +1251,13 @@
         <v>36</v>
       </c>
       <c r="N6" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="7" spans="1:15" s="3" customFormat="1" ht="60">
       <c r="A7" s="4" t="s">
         <v>141</v>
       </c>
@@ -1265,7 +1265,7 @@
         <v>102</v>
       </c>
       <c r="C7" s="5">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>15</v>
@@ -1274,7 +1274,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>140</v>
@@ -1298,13 +1298,13 @@
         <v>38</v>
       </c>
       <c r="N7" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O7" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="8" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A8" s="4" t="s">
         <v>141</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>102</v>
       </c>
       <c r="C8" s="5">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
@@ -1321,7 +1321,7 @@
         <v>36</v>
       </c>
       <c r="F8" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>139</v>
@@ -1341,13 +1341,13 @@
         <v>21</v>
       </c>
       <c r="N8" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O8" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="9" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A9" s="4" t="s">
         <v>141</v>
       </c>
@@ -1355,7 +1355,7 @@
         <v>102</v>
       </c>
       <c r="C9" s="5">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>15</v>
@@ -1364,7 +1364,7 @@
         <v>28</v>
       </c>
       <c r="F9" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>139</v>
@@ -1384,13 +1384,13 @@
         <v>36</v>
       </c>
       <c r="N9" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O9" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="10" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A10" s="4" t="s">
         <v>141</v>
       </c>
@@ -1398,7 +1398,7 @@
         <v>102</v>
       </c>
       <c r="C10" s="5">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>15</v>
@@ -1407,7 +1407,7 @@
         <v>38</v>
       </c>
       <c r="F10" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>139</v>
@@ -1427,13 +1427,13 @@
         <v>36</v>
       </c>
       <c r="N10" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O10" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="11" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A11" s="4" t="s">
         <v>141</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>102</v>
       </c>
       <c r="C11" s="5">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>15</v>
@@ -1450,7 +1450,7 @@
         <v>21</v>
       </c>
       <c r="F11" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>139</v>
@@ -1470,13 +1470,13 @@
         <v>36</v>
       </c>
       <c r="N11" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O11" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="12" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A12" s="4" t="s">
         <v>141</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>102</v>
       </c>
       <c r="C12" s="5">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>15</v>
@@ -1493,7 +1493,7 @@
         <v>36</v>
       </c>
       <c r="F12" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>139</v>
@@ -1513,13 +1513,13 @@
         <v>36</v>
       </c>
       <c r="N12" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O12" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="13" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A13" s="4" t="s">
         <v>141</v>
       </c>
@@ -1527,7 +1527,7 @@
         <v>102</v>
       </c>
       <c r="C13" s="5">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>15</v>
@@ -1536,7 +1536,7 @@
         <v>28</v>
       </c>
       <c r="F13" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>139</v>
@@ -1556,13 +1556,13 @@
         <v>21</v>
       </c>
       <c r="N13" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O13" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="14" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A14" s="4" t="s">
         <v>141</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>102</v>
       </c>
       <c r="C14" s="5">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>15</v>
@@ -1579,7 +1579,7 @@
         <v>38</v>
       </c>
       <c r="F14" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>139</v>
@@ -1599,13 +1599,13 @@
         <v>36</v>
       </c>
       <c r="N14" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O14" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="15" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A15" s="4" t="s">
         <v>141</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>102</v>
       </c>
       <c r="C15" s="5">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>15</v>
@@ -1622,7 +1622,7 @@
         <v>21</v>
       </c>
       <c r="F15" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>139</v>
@@ -1642,13 +1642,13 @@
         <v>36</v>
       </c>
       <c r="N15" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O15" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="8:8" s="3" ht="24.0" customFormat="1" customHeight="1">
+    <row r="16" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A16" s="4" t="s">
         <v>141</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>102</v>
       </c>
       <c r="C16" s="5">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>15</v>
@@ -1665,7 +1665,7 @@
         <v>28</v>
       </c>
       <c r="F16" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>139</v>
@@ -1685,13 +1685,13 @@
         <v>36</v>
       </c>
       <c r="N16" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O16" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="8:8" s="3" ht="24.0" customFormat="1" customHeight="1">
+    <row r="17" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A17" s="4" t="s">
         <v>141</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>102</v>
       </c>
       <c r="C17" s="5">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>15</v>
@@ -1708,7 +1708,7 @@
         <v>38</v>
       </c>
       <c r="F17" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>139</v>
@@ -1728,13 +1728,13 @@
         <v>36</v>
       </c>
       <c r="N17" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O17" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="8:8" s="3" ht="24.0" customFormat="1" customHeight="1">
+    <row r="18" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A18" s="4" t="s">
         <v>141</v>
       </c>
@@ -1742,7 +1742,7 @@
         <v>102</v>
       </c>
       <c r="C18" s="5">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>15</v>
@@ -1751,7 +1751,7 @@
         <v>36</v>
       </c>
       <c r="F18" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>139</v>
@@ -1771,13 +1771,13 @@
         <v>21</v>
       </c>
       <c r="N18" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O18" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="8:8" s="3" ht="24.0" customFormat="1" customHeight="1">
+    <row r="19" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A19" s="4" t="s">
         <v>141</v>
       </c>
@@ -1785,7 +1785,7 @@
         <v>102</v>
       </c>
       <c r="C19" s="5">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>15</v>
@@ -1794,7 +1794,7 @@
         <v>38</v>
       </c>
       <c r="F19" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>139</v>
@@ -1814,13 +1814,13 @@
         <v>36</v>
       </c>
       <c r="N19" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O19" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="20" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A20" s="4" t="s">
         <v>141</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>102</v>
       </c>
       <c r="C20" s="5">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>15</v>
@@ -1837,7 +1837,7 @@
         <v>28</v>
       </c>
       <c r="F20" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>140</v>
@@ -1861,13 +1861,13 @@
         <v>21</v>
       </c>
       <c r="N20" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O20" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="21" spans="1:15" s="3" customFormat="1" ht="45">
       <c r="A21" s="4" t="s">
         <v>141</v>
       </c>
@@ -1875,7 +1875,7 @@
         <v>102</v>
       </c>
       <c r="C21" s="5">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>15</v>
@@ -1884,7 +1884,7 @@
         <v>21</v>
       </c>
       <c r="F21" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>140</v>
@@ -1908,13 +1908,13 @@
         <v>36</v>
       </c>
       <c r="N21" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O21" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="22" spans="1:15" s="3" customFormat="1" ht="60">
       <c r="A22" s="4" t="s">
         <v>141</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>102</v>
       </c>
       <c r="C22" s="5">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>15</v>
@@ -1931,7 +1931,7 @@
         <v>38</v>
       </c>
       <c r="F22" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>140</v>
@@ -1955,13 +1955,13 @@
         <v>28</v>
       </c>
       <c r="N22" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O22" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="23" spans="1:15" s="3" customFormat="1" ht="45">
       <c r="A23" s="4" t="s">
         <v>141</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>102</v>
       </c>
       <c r="C23" s="5">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>15</v>
@@ -1978,7 +1978,7 @@
         <v>36</v>
       </c>
       <c r="F23" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>140</v>
@@ -2002,13 +2002,13 @@
         <v>38</v>
       </c>
       <c r="N23" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O23" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="24" spans="1:15" s="3" customFormat="1" ht="45">
       <c r="A24" s="4" t="s">
         <v>141</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>102</v>
       </c>
       <c r="C24" s="5">
-        <v>23.0</v>
+        <v>23</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>15</v>
@@ -2025,7 +2025,7 @@
         <v>38</v>
       </c>
       <c r="F24" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>140</v>
@@ -2049,13 +2049,13 @@
         <v>21</v>
       </c>
       <c r="N24" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O24" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="25" spans="1:15" s="3" customFormat="1" ht="45">
       <c r="A25" s="4" t="s">
         <v>141</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>102</v>
       </c>
       <c r="C25" s="5">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>15</v>
@@ -2072,7 +2072,7 @@
         <v>28</v>
       </c>
       <c r="F25" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>140</v>
@@ -2096,13 +2096,13 @@
         <v>28</v>
       </c>
       <c r="N25" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O25" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="26" spans="1:15" s="3" customFormat="1" ht="45">
       <c r="A26" s="4" t="s">
         <v>141</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>102</v>
       </c>
       <c r="C26" s="5">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>15</v>
@@ -2119,7 +2119,7 @@
         <v>21</v>
       </c>
       <c r="F26" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>140</v>
@@ -2143,13 +2143,13 @@
         <v>28</v>
       </c>
       <c r="N26" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O26" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="27" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A27" s="4" t="s">
         <v>141</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>102</v>
       </c>
       <c r="C27" s="5">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>15</v>
@@ -2166,7 +2166,7 @@
         <v>38</v>
       </c>
       <c r="F27" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>140</v>
@@ -2190,13 +2190,13 @@
         <v>38</v>
       </c>
       <c r="N27" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O27" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="28" spans="1:15" s="3" customFormat="1" ht="30">
       <c r="A28" s="4" t="s">
         <v>141</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>102</v>
       </c>
       <c r="C28" s="5">
-        <v>27.0</v>
+        <v>27</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>15</v>
@@ -2213,7 +2213,7 @@
         <v>36</v>
       </c>
       <c r="F28" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>139</v>
@@ -2233,13 +2233,13 @@
         <v>21</v>
       </c>
       <c r="N28" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O28" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="29" spans="1:15" s="3" customFormat="1">
       <c r="A29" s="4" t="s">
         <v>141</v>
       </c>
@@ -2247,7 +2247,7 @@
         <v>102</v>
       </c>
       <c r="C29" s="5">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>15</v>
@@ -2256,7 +2256,7 @@
         <v>38</v>
       </c>
       <c r="F29" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>140</v>
@@ -2280,13 +2280,13 @@
         <v>36</v>
       </c>
       <c r="N29" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O29" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="30" spans="1:15" s="3" customFormat="1">
       <c r="A30" s="4" t="s">
         <v>141</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>102</v>
       </c>
       <c r="C30" s="5">
-        <v>29.0</v>
+        <v>29</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>15</v>
@@ -2303,7 +2303,7 @@
         <v>36</v>
       </c>
       <c r="F30" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>139</v>
@@ -2323,13 +2323,13 @@
         <v>36</v>
       </c>
       <c r="N30" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O30" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="31" spans="1:15" s="3" customFormat="1">
       <c r="A31" s="4" t="s">
         <v>141</v>
       </c>
@@ -2337,7 +2337,7 @@
         <v>102</v>
       </c>
       <c r="C31" s="5">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>15</v>
@@ -2346,7 +2346,7 @@
         <v>28</v>
       </c>
       <c r="F31" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>140</v>
@@ -2370,13 +2370,13 @@
         <v>21</v>
       </c>
       <c r="N31" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O31" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="32" spans="1:15" s="3" customFormat="1">
       <c r="A32" s="4" t="s">
         <v>141</v>
       </c>
@@ -2384,7 +2384,7 @@
         <v>102</v>
       </c>
       <c r="C32" s="5">
-        <v>31.0</v>
+        <v>31</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>15</v>
@@ -2393,7 +2393,7 @@
         <v>36</v>
       </c>
       <c r="F32" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>140</v>
@@ -2417,13 +2417,13 @@
         <v>38</v>
       </c>
       <c r="N32" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O32" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="33" spans="1:15" s="3" customFormat="1">
       <c r="A33" s="4" t="s">
         <v>141</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>102</v>
       </c>
       <c r="C33" s="5">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>15</v>
@@ -2440,7 +2440,7 @@
         <v>36</v>
       </c>
       <c r="F33" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>140</v>
@@ -2464,13 +2464,13 @@
         <v>38</v>
       </c>
       <c r="N33" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O33" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="34" spans="1:15" s="3" customFormat="1">
       <c r="A34" s="4" t="s">
         <v>141</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>102</v>
       </c>
       <c r="C34" s="5">
-        <v>33.0</v>
+        <v>33</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>15</v>
@@ -2487,7 +2487,7 @@
         <v>28</v>
       </c>
       <c r="F34" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>140</v>
@@ -2511,13 +2511,13 @@
         <v>28</v>
       </c>
       <c r="N34" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O34" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="35" spans="1:15" s="3" customFormat="1">
       <c r="A35" s="4" t="s">
         <v>141</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>102</v>
       </c>
       <c r="C35" s="5">
-        <v>34.0</v>
+        <v>34</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>15</v>
@@ -2534,7 +2534,7 @@
         <v>36</v>
       </c>
       <c r="F35" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>139</v>
@@ -2554,13 +2554,13 @@
         <v>21</v>
       </c>
       <c r="N35" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O35" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="36" spans="1:15" s="3" customFormat="1">
       <c r="A36" s="4" t="s">
         <v>141</v>
       </c>
@@ -2568,7 +2568,7 @@
         <v>102</v>
       </c>
       <c r="C36" s="5">
-        <v>35.0</v>
+        <v>35</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>15</v>
@@ -2577,7 +2577,7 @@
         <v>36</v>
       </c>
       <c r="F36" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>139</v>
@@ -2597,13 +2597,13 @@
         <v>36</v>
       </c>
       <c r="N36" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O36" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="8:8" s="3" ht="75.0" customFormat="1">
+    <row r="37" spans="1:15" s="3" customFormat="1">
       <c r="A37" s="4" t="s">
         <v>141</v>
       </c>
@@ -2611,7 +2611,7 @@
         <v>102</v>
       </c>
       <c r="C37" s="5">
-        <v>36.0</v>
+        <v>36</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>15</v>
@@ -2620,7 +2620,7 @@
         <v>21</v>
       </c>
       <c r="F37" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>139</v>
@@ -2640,13 +2640,13 @@
         <v>36</v>
       </c>
       <c r="N37" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="O37" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="8:8" ht="75.0">
+    <row r="38" spans="1:15" ht="60">
       <c r="A38" s="4" t="s">
         <v>141</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>102</v>
       </c>
       <c r="C38" s="5">
-        <v>37.0</v>
+        <v>37</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>15</v>
@@ -2663,7 +2663,7 @@
         <v>21</v>
       </c>
       <c r="F38" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>140</v>
@@ -2687,13 +2687,13 @@
         <v>36</v>
       </c>
       <c r="N38" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O38" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="39" spans="8:8" ht="75.0">
+    <row r="39" spans="1:15" ht="30">
       <c r="A39" s="4" t="s">
         <v>141</v>
       </c>
@@ -2701,7 +2701,7 @@
         <v>102</v>
       </c>
       <c r="C39" s="5">
-        <v>38.0</v>
+        <v>38</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>15</v>
@@ -2710,7 +2710,7 @@
         <v>36</v>
       </c>
       <c r="F39" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>140</v>
@@ -2734,13 +2734,13 @@
         <v>28</v>
       </c>
       <c r="N39" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="40" spans="8:8" ht="75.0">
+    <row r="40" spans="1:15" ht="30">
       <c r="A40" s="4" t="s">
         <v>141</v>
       </c>
@@ -2748,7 +2748,7 @@
         <v>102</v>
       </c>
       <c r="C40" s="5">
-        <v>39.0</v>
+        <v>39</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>15</v>
@@ -2757,7 +2757,7 @@
         <v>38</v>
       </c>
       <c r="F40" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>140</v>
@@ -2781,13 +2781,13 @@
         <v>36</v>
       </c>
       <c r="N40" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O40" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="41" spans="8:8" ht="75.0">
+    <row r="41" spans="1:15" ht="30">
       <c r="A41" s="4" t="s">
         <v>141</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>102</v>
       </c>
       <c r="C41" s="5">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>15</v>
@@ -2804,7 +2804,7 @@
         <v>38</v>
       </c>
       <c r="F41" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>140</v>
@@ -2828,13 +2828,13 @@
         <v>21</v>
       </c>
       <c r="N41" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O41" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="42" spans="8:8" ht="75.0">
+    <row r="42" spans="1:15" ht="30">
       <c r="A42" s="4" t="s">
         <v>141</v>
       </c>
@@ -2842,7 +2842,7 @@
         <v>102</v>
       </c>
       <c r="C42" s="5">
-        <v>41.0</v>
+        <v>41</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>15</v>
@@ -2851,7 +2851,7 @@
         <v>36</v>
       </c>
       <c r="F42" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>140</v>
@@ -2875,13 +2875,13 @@
         <v>36</v>
       </c>
       <c r="N42" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O42" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="43" spans="8:8" ht="75.0">
+    <row r="43" spans="1:15">
       <c r="A43" s="4" t="s">
         <v>141</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>102</v>
       </c>
       <c r="C43" s="5">
-        <v>42.0</v>
+        <v>42</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>15</v>
@@ -2898,7 +2898,7 @@
         <v>28</v>
       </c>
       <c r="F43" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G43" s="5" t="s">
         <v>140</v>
@@ -2922,13 +2922,13 @@
         <v>38</v>
       </c>
       <c r="N43" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O43" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="8:8" ht="75.0">
+    <row r="44" spans="1:15" ht="30">
       <c r="A44" s="4" t="s">
         <v>141</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>102</v>
       </c>
       <c r="C44" s="5">
-        <v>43.0</v>
+        <v>43</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>15</v>
@@ -2945,7 +2945,7 @@
         <v>21</v>
       </c>
       <c r="F44" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>140</v>
@@ -2969,13 +2969,13 @@
         <v>28</v>
       </c>
       <c r="N44" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O44" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="45" spans="8:8" ht="75.0">
+    <row r="45" spans="1:15" ht="30">
       <c r="A45" s="4" t="s">
         <v>141</v>
       </c>
@@ -2983,7 +2983,7 @@
         <v>102</v>
       </c>
       <c r="C45" s="5">
-        <v>44.0</v>
+        <v>44</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>15</v>
@@ -2992,7 +2992,7 @@
         <v>36</v>
       </c>
       <c r="F45" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>140</v>
@@ -3016,13 +3016,13 @@
         <v>36</v>
       </c>
       <c r="N45" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O45" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="46" spans="8:8" ht="75.0">
+    <row r="46" spans="1:15" ht="30">
       <c r="A46" s="4" t="s">
         <v>141</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>102</v>
       </c>
       <c r="C46" s="5">
-        <v>45.0</v>
+        <v>45</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>15</v>
@@ -3039,7 +3039,7 @@
         <v>38</v>
       </c>
       <c r="F46" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>140</v>
@@ -3063,13 +3063,13 @@
         <v>28</v>
       </c>
       <c r="N46" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O46" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="8:8" ht="75.0" customFormat="1">
+    <row r="47" spans="1:15" ht="30">
       <c r="A47" s="8" t="s">
         <v>142</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>102</v>
       </c>
       <c r="C47" s="5">
-        <v>46.0</v>
+        <v>46</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>15</v>
@@ -3086,7 +3086,7 @@
         <v>38</v>
       </c>
       <c r="F47" s="4">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G47" s="4" t="s">
         <v>140</v>
@@ -3110,13 +3110,13 @@
         <v>36</v>
       </c>
       <c r="N47" s="4">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O47" s="4" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="8:8" ht="75.0" customFormat="1">
+    <row r="48" spans="1:15" ht="30">
       <c r="A48" s="8" t="s">
         <v>142</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>102</v>
       </c>
       <c r="C48" s="5">
-        <v>47.0</v>
+        <v>47</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>15</v>
@@ -3133,7 +3133,7 @@
         <v>28</v>
       </c>
       <c r="F48" s="4">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G48" s="4" t="s">
         <v>140</v>
@@ -3157,7 +3157,7 @@
         <v>38</v>
       </c>
       <c r="N48" s="4">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="O48" s="4" t="s">
         <v>138</v>
@@ -3165,28 +3165,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H1">
-    <cfRule type="duplicateValues" priority="3" dxfId="0"/>
-    <cfRule type="duplicateValues" priority="2" dxfId="1"/>
-    <cfRule type="duplicateValues" priority="6" dxfId="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="6"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15.0" defaultColWidth="10"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15.0" defaultColWidth="10"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>